<commit_message>
add cookie-based session auth for GET attendance
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -539,7 +539,7 @@
     <col min="1" max="1" style="10" width="22.005" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="11" width="22.005" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="11" width="22.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="13" width="25.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="42.005" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="11" width="22.005" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="11" width="22.005" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="13" width="22.005" customWidth="1" bestFit="1"/>
@@ -570,7 +570,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="3">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
Playwright soft expect added to log failure
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,13 +426,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>01/17/2026</v>
+        <v>03/15/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>09:00 AM</v>
+        <v>10:30 AM</v>
       </c>
       <c r="C2" t="str">
-        <v>05:00 PM</v>
+        <v>10:30 AM</v>
       </c>
       <c r="D2" t="str">
         <v>BS-MIRNY-Q6P4N5XGUMULE</v>
@@ -449,13 +449,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>01/18/2026</v>
+        <v>03/16/2026</v>
       </c>
       <c r="B3" t="str">
         <v>10:30 AM</v>
       </c>
       <c r="C3" t="str">
-        <v>11:30 AM</v>
+        <v>10:30 AM</v>
       </c>
       <c r="D3" t="str">
         <v>BS-MIRNY-Q6P4N5XGUMULE</v>
@@ -470,9 +470,129 @@
         <v>Short Session Check</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>03/17/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="C4" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BS-MIRNY-Q6P4N5XGUMULE</v>
+      </c>
+      <c r="E4" t="str">
+        <v>P</v>
+      </c>
+      <c r="F4" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Short Session Check</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>03/18/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="C5" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="D5" t="str">
+        <v>BS-MIRNY-Q6P4N5XGUMULE</v>
+      </c>
+      <c r="E5" t="str">
+        <v>P</v>
+      </c>
+      <c r="F5" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Short Session Check</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>03/19/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="C6" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="D6" t="str">
+        <v>BS-MIRNY-Q6P4N5XGUMULE</v>
+      </c>
+      <c r="E6" t="str">
+        <v>P</v>
+      </c>
+      <c r="F6" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Short Session Check</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>03/20/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="C7" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="D7" t="str">
+        <v>BS-MIRNY-Q6P4N5XGUMULE</v>
+      </c>
+      <c r="E7" t="str">
+        <v>P</v>
+      </c>
+      <c r="F7" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Short Session Check</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>03/21/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="C8" t="str">
+        <v>10:30 AM</v>
+      </c>
+      <c r="D8" t="str">
+        <v>BS-MIRNY-Q6P4N5XGUMULE</v>
+      </c>
+      <c r="E8" t="str">
+        <v>P</v>
+      </c>
+      <c r="F8" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Short Session Check</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>03/21/2027</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -540,7 +660,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>46039</v>
+        <v>46133</v>
       </c>
       <c r="B2" t="str">
         <v>09:00 AM</v>
@@ -563,7 +683,7 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>46040</v>
+        <v>46134</v>
       </c>
       <c r="B3" t="str">
         <v>10:30 AM</v>
@@ -586,7 +706,7 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>46041</v>
+        <v>46135</v>
       </c>
       <c r="B4" t="str">
         <v>02:00 PM</v>
@@ -609,7 +729,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>46042</v>
+        <v>46136</v>
       </c>
       <c r="B5" t="str">
         <v>11:00 PM</v>
@@ -632,7 +752,7 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>46043</v>
+        <v>46137</v>
       </c>
       <c r="D6" t="str">
         <v>BS-MIRNY-Q6P4N5XGUMULE</v>
@@ -646,7 +766,7 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>46044</v>
+        <v>46138</v>
       </c>
       <c r="B7" t="str">
         <v>11:00 PM</v>
@@ -669,7 +789,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>46045</v>
+        <v>46139</v>
       </c>
       <c r="B8" t="str">
         <v>11:00 PM</v>
@@ -689,7 +809,7 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>46046</v>
+        <v>46140</v>
       </c>
       <c r="B9" t="str">
         <v>11:00 PM</v>
@@ -712,7 +832,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>46047</v>
+        <v>46141</v>
       </c>
       <c r="B10" t="str">
         <v>11:00 PM</v>
@@ -735,7 +855,7 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>46048</v>
+        <v>46142</v>
       </c>
       <c r="B11" t="str">
         <v>11:00 PM</v>
@@ -754,8 +874,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
-        <v>04/21/26'</v>
+      <c r="A12">
+        <v>46143</v>
       </c>
       <c r="B12" t="str">
         <v>11:00 PM</v>

</xml_diff>

<commit_message>
Forcing TherapClient.js into repo
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -426,7 +426,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>03/15/2026</v>
+        <v>03/23/2026</v>
       </c>
       <c r="B2" t="str">
         <v>10:30 AM</v>
@@ -449,7 +449,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>03/16/2026</v>
+        <v>03/24/2026</v>
       </c>
       <c r="B3" t="str">
         <v>10:30 AM</v>
@@ -472,7 +472,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>03/17/2026</v>
+        <v>03/25/2026</v>
       </c>
       <c r="B4" t="str">
         <v>10:30 AM</v>
@@ -495,7 +495,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>03/18/2026</v>
+        <v>03/26/2026</v>
       </c>
       <c r="B5" t="str">
         <v>10:30 AM</v>
@@ -518,7 +518,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>03/19/2026</v>
+        <v>03/27/2026</v>
       </c>
       <c r="B6" t="str">
         <v>10:30 AM</v>
@@ -541,7 +541,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>03/20/2026</v>
+        <v>03/28/2026</v>
       </c>
       <c r="B7" t="str">
         <v>10:30 AM</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>03/21/2026</v>
+        <v>03/29/2026</v>
       </c>
       <c r="B8" t="str">
         <v>10:30 AM</v>
@@ -587,7 +587,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>03/21/2027</v>
+        <v>03/29/2027</v>
       </c>
     </row>
   </sheetData>

</xml_diff>